<commit_message>
Add Recommended Price Summary sheet (one best price per workshop)
New front sheet listing a single headline recommended price for each of
the 27 workshops (the full premium workshop), with market median for
reference and a portfolio total. Complements the 3-tier breakdown sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjvYXygDKkAN1X1SuAqsBh
</commit_message>
<xml_diff>
--- a/SGMB_Pricing_With_Recommendations.xlsx
+++ b/SGMB_Pricing_With_Recommendations.xlsx
@@ -7,14 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SGMB Pricing Recommendation" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Benchmark Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes &amp; Gaps" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary by Category" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Workshop Index" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Recommended Price Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SGMB Pricing Recommendation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Benchmark Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes &amp; Gaps" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary by Category" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Workshop Index" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Benchmark Data'!$A$3:$N$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Benchmark Data'!$A$3:$N$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -229,7 +230,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -266,6 +267,50 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -277,7 +322,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -487,6 +532,14 @@
     <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -758,6 +811,704 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" style="27" min="1" max="1"/>
+    <col width="40" customWidth="1" style="27" min="2" max="2"/>
+    <col width="28" customWidth="1" style="27" min="3" max="3"/>
+    <col width="18" customWidth="1" style="27" min="4" max="4"/>
+    <col width="22" customWidth="1" style="27" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>SGMB Recommended Price — Best Single Price per Workshop</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="56" customHeight="1" s="27">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>One headline price per workshop = the complete premium workshop (multi-day, government-quality). Positioned at the upper-mid of the market (~60th percentile of confirmed competitor prices, above median, capped at the 90th percentile). Prices in AED, exclude 5% VAT. USD 1=3.67 / EUR 1=4.07 AED. See "SGMB Pricing Recommendation" sheet for Online / One-Day / Full Course tier breakdown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1" s="27">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>SGMB Code</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>Workshop Name</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>Market Median (AED)</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Recommended Price (AED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="42" t="inlineStr">
+        <is>
+          <t>W01</t>
+        </is>
+      </c>
+      <c r="B5" s="43" t="inlineStr">
+        <is>
+          <t>Media Communication Fundamentals</t>
+        </is>
+      </c>
+      <c r="C5" s="43" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism</t>
+        </is>
+      </c>
+      <c r="D5" s="44" t="n">
+        <v>10826</v>
+      </c>
+      <c r="E5" s="41" t="n">
+        <v>13750</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="36" t="inlineStr">
+        <is>
+          <t>W02</t>
+        </is>
+      </c>
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>Digital Journalism</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="n">
+        <v>5505</v>
+      </c>
+      <c r="E6" s="41" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="42" t="inlineStr">
+        <is>
+          <t>W03</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="inlineStr">
+        <is>
+          <t>TV Reporting</t>
+        </is>
+      </c>
+      <c r="C7" s="43" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism</t>
+        </is>
+      </c>
+      <c r="D7" s="44" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E7" s="41" t="n">
+        <v>5250</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>W04</t>
+        </is>
+      </c>
+      <c r="B8" s="37" t="inlineStr">
+        <is>
+          <t>Job Interview Track</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="n">
+        <v>6591</v>
+      </c>
+      <c r="E8" s="41" t="n">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="42" t="inlineStr">
+        <is>
+          <t>W05</t>
+        </is>
+      </c>
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>Art of Management</t>
+        </is>
+      </c>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="n">
+        <v>13671</v>
+      </c>
+      <c r="E9" s="41" t="n">
+        <v>14500</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="36" t="inlineStr">
+        <is>
+          <t>W06</t>
+        </is>
+      </c>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Journalistic Workshop</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="n">
+        <v>3745</v>
+      </c>
+      <c r="E10" s="41" t="n">
+        <v>4300</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="42" t="inlineStr">
+        <is>
+          <t>W07</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="inlineStr">
+        <is>
+          <t>International Forums Organization</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>Events &amp; Protocol</t>
+        </is>
+      </c>
+      <c r="D11" s="44" t="n">
+        <v>4300</v>
+      </c>
+      <c r="E11" s="41" t="n">
+        <v>11750</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="36" t="inlineStr">
+        <is>
+          <t>W08</t>
+        </is>
+      </c>
+      <c r="B12" s="37" t="inlineStr">
+        <is>
+          <t>Official Email Correspondence</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="n">
+        <v>9359</v>
+      </c>
+      <c r="E12" s="41" t="n">
+        <v>10750</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="42" t="inlineStr">
+        <is>
+          <t>W09</t>
+        </is>
+      </c>
+      <c r="B13" s="43" t="inlineStr">
+        <is>
+          <t>Event Management</t>
+        </is>
+      </c>
+      <c r="C13" s="43" t="inlineStr">
+        <is>
+          <t>Events &amp; Protocol</t>
+        </is>
+      </c>
+      <c r="D13" s="44" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E13" s="41" t="n">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>Ceremonies &amp; Protocol</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>Events &amp; Protocol</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="n">
+        <v>20001</v>
+      </c>
+      <c r="E14" s="41" t="n">
+        <v>21750</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="42" t="inlineStr">
+        <is>
+          <t>W11</t>
+        </is>
+      </c>
+      <c r="B15" s="43" t="inlineStr">
+        <is>
+          <t>Social Media Coverage</t>
+        </is>
+      </c>
+      <c r="C15" s="43" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital</t>
+        </is>
+      </c>
+      <c r="D15" s="44" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E15" s="41" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="36" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="B16" s="37" t="inlineStr">
+        <is>
+          <t>Photojournalism &amp; Photography</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>Design &amp; Photography</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="n">
+        <v>648</v>
+      </c>
+      <c r="E16" s="41" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="B17" s="43" t="inlineStr">
+        <is>
+          <t>Portrait Photography</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>Design &amp; Photography</t>
+        </is>
+      </c>
+      <c r="D17" s="44" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E17" s="41" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="36" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>Story Telling Workshop</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism</t>
+        </is>
+      </c>
+      <c r="D18" s="38" t="n">
+        <v>9359</v>
+      </c>
+      <c r="E18" s="41" t="n">
+        <v>10750</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="42" t="inlineStr">
+        <is>
+          <t>W15</t>
+        </is>
+      </c>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>Media Coverage</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism</t>
+        </is>
+      </c>
+      <c r="D19" s="44" t="n">
+        <v>15781</v>
+      </c>
+      <c r="E19" s="41" t="n">
+        <v>17000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="36" t="inlineStr">
+        <is>
+          <t>W16</t>
+        </is>
+      </c>
+      <c r="B20" s="37" t="inlineStr">
+        <is>
+          <t>Law in the Workplace</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="D20" s="38" t="n">
+        <v>634</v>
+      </c>
+      <c r="E20" s="41" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="42" t="inlineStr">
+        <is>
+          <t>W17</t>
+        </is>
+      </c>
+      <c r="B21" s="43" t="inlineStr">
+        <is>
+          <t>Creative Thinking in the Workplace</t>
+        </is>
+      </c>
+      <c r="C21" s="43" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional</t>
+        </is>
+      </c>
+      <c r="D21" s="44" t="n">
+        <v>6588</v>
+      </c>
+      <c r="E21" s="41" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="36" t="inlineStr">
+        <is>
+          <t>W18</t>
+        </is>
+      </c>
+      <c r="B22" s="37" t="inlineStr">
+        <is>
+          <t>TV Directing</t>
+        </is>
+      </c>
+      <c r="C22" s="37" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism</t>
+        </is>
+      </c>
+      <c r="D22" s="38" t="n">
+        <v>4250</v>
+      </c>
+      <c r="E22" s="41" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="42" t="inlineStr">
+        <is>
+          <t>W19</t>
+        </is>
+      </c>
+      <c r="B23" s="43" t="inlineStr">
+        <is>
+          <t>TV Editing / Montage</t>
+        </is>
+      </c>
+      <c r="C23" s="43" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism</t>
+        </is>
+      </c>
+      <c r="D23" s="44" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E23" s="41" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="36" t="inlineStr">
+        <is>
+          <t>W20</t>
+        </is>
+      </c>
+      <c r="B24" s="37" t="inlineStr">
+        <is>
+          <t>Verifying Information on Social Media</t>
+        </is>
+      </c>
+      <c r="C24" s="37" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital</t>
+        </is>
+      </c>
+      <c r="D24" s="38" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E24" s="41" t="n">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="42" t="inlineStr">
+        <is>
+          <t>W21</t>
+        </is>
+      </c>
+      <c r="B25" s="43" t="inlineStr">
+        <is>
+          <t>Social Media Graphic Design &amp; Coordination</t>
+        </is>
+      </c>
+      <c r="C25" s="43" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital</t>
+        </is>
+      </c>
+      <c r="D25" s="44" t="n">
+        <v>2150</v>
+      </c>
+      <c r="E25" s="41" t="n">
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t>W22</t>
+        </is>
+      </c>
+      <c r="B26" s="37" t="inlineStr">
+        <is>
+          <t>Graphic Design</t>
+        </is>
+      </c>
+      <c r="C26" s="37" t="inlineStr">
+        <is>
+          <t>Design &amp; Photography</t>
+        </is>
+      </c>
+      <c r="D26" s="38" t="n">
+        <v>1550</v>
+      </c>
+      <c r="E26" s="41" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>W23</t>
+        </is>
+      </c>
+      <c r="B27" s="43" t="inlineStr">
+        <is>
+          <t>Strategic Communication</t>
+        </is>
+      </c>
+      <c r="C27" s="43" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital</t>
+        </is>
+      </c>
+      <c r="D27" s="44" t="n">
+        <v>4600</v>
+      </c>
+      <c r="E27" s="41" t="n">
+        <v>5500</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="36" t="inlineStr">
+        <is>
+          <t>W24</t>
+        </is>
+      </c>
+      <c r="B28" s="37" t="inlineStr">
+        <is>
+          <t>Website Content Management</t>
+        </is>
+      </c>
+      <c r="C28" s="37" t="inlineStr">
+        <is>
+          <t>Technology &amp; Cybersecurity</t>
+        </is>
+      </c>
+      <c r="D28" s="38" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E28" s="41" t="n">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t>W25</t>
+        </is>
+      </c>
+      <c r="B29" s="43" t="inlineStr">
+        <is>
+          <t>Financial Budgets</t>
+        </is>
+      </c>
+      <c r="C29" s="43" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional</t>
+        </is>
+      </c>
+      <c r="D29" s="44" t="n">
+        <v>15793</v>
+      </c>
+      <c r="E29" s="41" t="n">
+        <v>18250</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
+        <is>
+          <t>W26</t>
+        </is>
+      </c>
+      <c r="B30" s="37" t="inlineStr">
+        <is>
+          <t>Computer Applications Skills</t>
+        </is>
+      </c>
+      <c r="C30" s="37" t="inlineStr">
+        <is>
+          <t>Technology &amp; Cybersecurity</t>
+        </is>
+      </c>
+      <c r="D30" s="38" t="n">
+        <v>1675</v>
+      </c>
+      <c r="E30" s="41" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="42" t="inlineStr">
+        <is>
+          <t>W27</t>
+        </is>
+      </c>
+      <c r="B31" s="43" t="inlineStr">
+        <is>
+          <t>Cybersecurity &amp; Protection from Hacking</t>
+        </is>
+      </c>
+      <c r="C31" s="43" t="inlineStr">
+        <is>
+          <t>Technology &amp; Cybersecurity</t>
+        </is>
+      </c>
+      <c r="D31" s="44" t="n">
+        <v>2810</v>
+      </c>
+      <c r="E31" s="41" t="n">
+        <v>3100</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="71" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E32" s="72" t="n">
+        <v>184500</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A32:D32"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -794,22 +1545,22 @@
           <t>WORKSHOP</t>
         </is>
       </c>
-      <c r="B4" s="30" t="n"/>
-      <c r="C4" s="30" t="n"/>
+      <c r="B4" s="73" t="n"/>
+      <c r="C4" s="74" t="n"/>
       <c r="D4" s="31" t="inlineStr">
         <is>
           <t>COMPETITOR MARKET (AED)</t>
         </is>
       </c>
-      <c r="E4" s="31" t="n"/>
-      <c r="F4" s="31" t="n"/>
+      <c r="E4" s="73" t="n"/>
+      <c r="F4" s="74" t="n"/>
       <c r="G4" s="30" t="inlineStr">
         <is>
           <t>RECOMMENDED SGMB PRICE (AED)</t>
         </is>
       </c>
-      <c r="H4" s="30" t="n"/>
-      <c r="I4" s="30" t="n"/>
+      <c r="H4" s="73" t="n"/>
+      <c r="I4" s="74" t="n"/>
       <c r="J4" s="30" t="inlineStr"/>
       <c r="K4" s="30" t="inlineStr"/>
     </row>
@@ -1961,7 +2712,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12080,7 +12831,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14742,7 +15493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14989,7 +15740,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add Arabic workshop names to pricing sheets
Add bilingual (English + Arabic) workshop names to both the Recommended
Price Summary and SGMB Pricing Recommendation sheets, using the Arabic
names from the Workshop Index, with right-to-left alignment.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjvYXygDKkAN1X1SuAqsBh
</commit_message>
<xml_diff>
--- a/SGMB_Pricing_With_Recommendations.xlsx
+++ b/SGMB_Pricing_With_Recommendations.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -104,6 +104,24 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="23">
@@ -322,7 +340,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -540,6 +558,37 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -811,52 +860,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="27" min="1" max="1"/>
-    <col width="40" customWidth="1" style="27" min="2" max="2"/>
-    <col width="28" customWidth="1" style="27" min="3" max="3"/>
-    <col width="18" customWidth="1" style="27" min="4" max="4"/>
-    <col width="22" customWidth="1" style="27" min="5" max="5"/>
+    <col width="38" customWidth="1" style="27" min="2" max="2"/>
+    <col width="34" customWidth="1" style="27" min="3" max="3"/>
+    <col width="26" customWidth="1" style="27" min="4" max="4"/>
+    <col width="18" customWidth="1" style="27" min="5" max="5"/>
+    <col width="22" customWidth="1" style="27" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="28" t="inlineStr">
         <is>
-          <t>SGMB Recommended Price — Best Single Price per Workshop</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="56" customHeight="1" s="27">
+          <t>SGMB Recommended Price — Best Single Price per Workshop  |  السعر الموصى به لكل ورشة</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1" s="27">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>One headline price per workshop = the complete premium workshop (multi-day, government-quality). Positioned at the upper-mid of the market (~60th percentile of confirmed competitor prices, above median, capped at the 90th percentile). Prices in AED, exclude 5% VAT. USD 1=3.67 / EUR 1=4.07 AED. See "SGMB Pricing Recommendation" sheet for Online / One-Day / Full Course tier breakdown.</t>
+          <t>One headline price per workshop = the complete premium workshop (multi-day, government-quality), positioned at the upper-mid of the market. Prices in AED, exclude 5% VAT. السعر الموصى به لكل ورشة (الورشة الكاملة) بالدرهم الإماراتي، غير شامل ضريبة القيمة المضافة ٥٪.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="27">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="75" t="inlineStr">
         <is>
           <t>SGMB Code</t>
         </is>
       </c>
-      <c r="B4" s="30" t="inlineStr">
+      <c r="B4" s="75" t="inlineStr">
         <is>
           <t>Workshop Name</t>
         </is>
       </c>
-      <c r="C4" s="30" t="inlineStr">
+      <c r="C4" s="76" t="inlineStr">
+        <is>
+          <t>اسم الورشة</t>
+        </is>
+      </c>
+      <c r="D4" s="75" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D4" s="31" t="inlineStr">
+      <c r="E4" s="77" t="inlineStr">
         <is>
           <t>Market Median (AED)</t>
         </is>
       </c>
-      <c r="E4" s="35" t="inlineStr">
+      <c r="F4" s="78" t="inlineStr">
         <is>
           <t>Recommended Price (AED)</t>
         </is>
@@ -873,15 +928,20 @@
           <t>Media Communication Fundamentals</t>
         </is>
       </c>
-      <c r="C5" s="43" t="inlineStr">
+      <c r="C5" s="79" t="inlineStr">
+        <is>
+          <t>ورشة أصول التعامل الإعلامي</t>
+        </is>
+      </c>
+      <c r="D5" s="43" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D5" s="44" t="n">
+      <c r="E5" s="44" t="n">
         <v>10826</v>
       </c>
-      <c r="E5" s="41" t="n">
+      <c r="F5" s="41" t="n">
         <v>13750</v>
       </c>
     </row>
@@ -896,15 +956,20 @@
           <t>Digital Journalism</t>
         </is>
       </c>
-      <c r="C6" s="37" t="inlineStr">
+      <c r="C6" s="80" t="inlineStr">
+        <is>
+          <t>ورشة الصحافة الرقمية</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D6" s="38" t="n">
+      <c r="E6" s="38" t="n">
         <v>5505</v>
       </c>
-      <c r="E6" s="41" t="n">
+      <c r="F6" s="41" t="n">
         <v>6000</v>
       </c>
     </row>
@@ -919,15 +984,20 @@
           <t>TV Reporting</t>
         </is>
       </c>
-      <c r="C7" s="43" t="inlineStr">
+      <c r="C7" s="79" t="inlineStr">
+        <is>
+          <t>ورشة التقرير التلفزيوني</t>
+        </is>
+      </c>
+      <c r="D7" s="43" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D7" s="44" t="n">
+      <c r="E7" s="44" t="n">
         <v>5000</v>
       </c>
-      <c r="E7" s="41" t="n">
+      <c r="F7" s="41" t="n">
         <v>5250</v>
       </c>
     </row>
@@ -942,15 +1012,20 @@
           <t>Job Interview Track</t>
         </is>
       </c>
-      <c r="C8" s="37" t="inlineStr">
+      <c r="C8" s="80" t="inlineStr">
+        <is>
+          <t>ورشة مسار المقابلات الوظيفية</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
       </c>
-      <c r="D8" s="38" t="n">
+      <c r="E8" s="38" t="n">
         <v>6591</v>
       </c>
-      <c r="E8" s="41" t="n">
+      <c r="F8" s="41" t="n">
         <v>6500</v>
       </c>
     </row>
@@ -965,15 +1040,20 @@
           <t>Art of Management</t>
         </is>
       </c>
-      <c r="C9" s="43" t="inlineStr">
+      <c r="C9" s="79" t="inlineStr">
+        <is>
+          <t>ورشة فن الإدارة</t>
+        </is>
+      </c>
+      <c r="D9" s="43" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
       </c>
-      <c r="D9" s="44" t="n">
+      <c r="E9" s="44" t="n">
         <v>13671</v>
       </c>
-      <c r="E9" s="41" t="n">
+      <c r="F9" s="41" t="n">
         <v>14500</v>
       </c>
     </row>
@@ -988,15 +1068,20 @@
           <t>Journalistic Workshop</t>
         </is>
       </c>
-      <c r="C10" s="37" t="inlineStr">
+      <c r="C10" s="80" t="inlineStr">
+        <is>
+          <t>الورشة الصحفية</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D10" s="38" t="n">
+      <c r="E10" s="38" t="n">
         <v>3745</v>
       </c>
-      <c r="E10" s="41" t="n">
+      <c r="F10" s="41" t="n">
         <v>4300</v>
       </c>
     </row>
@@ -1011,15 +1096,20 @@
           <t>International Forums Organization</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="79" t="inlineStr">
+        <is>
+          <t>ورشة تنظيم المنتديات الدولية</t>
+        </is>
+      </c>
+      <c r="D11" s="43" t="inlineStr">
         <is>
           <t>Events &amp; Protocol</t>
         </is>
       </c>
-      <c r="D11" s="44" t="n">
+      <c r="E11" s="44" t="n">
         <v>4300</v>
       </c>
-      <c r="E11" s="41" t="n">
+      <c r="F11" s="41" t="n">
         <v>11750</v>
       </c>
     </row>
@@ -1034,15 +1124,20 @@
           <t>Official Email Correspondence</t>
         </is>
       </c>
-      <c r="C12" s="37" t="inlineStr">
+      <c r="C12" s="80" t="inlineStr">
+        <is>
+          <t>ورشة المخاطبات الرسمية بالبريد الإلكتروني</t>
+        </is>
+      </c>
+      <c r="D12" s="37" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
       </c>
-      <c r="D12" s="38" t="n">
+      <c r="E12" s="38" t="n">
         <v>9359</v>
       </c>
-      <c r="E12" s="41" t="n">
+      <c r="F12" s="41" t="n">
         <v>10750</v>
       </c>
     </row>
@@ -1057,15 +1152,20 @@
           <t>Event Management</t>
         </is>
       </c>
-      <c r="C13" s="43" t="inlineStr">
+      <c r="C13" s="79" t="inlineStr">
+        <is>
+          <t>ورشة تنظيم الفعاليات</t>
+        </is>
+      </c>
+      <c r="D13" s="43" t="inlineStr">
         <is>
           <t>Events &amp; Protocol</t>
         </is>
       </c>
-      <c r="D13" s="44" t="n">
+      <c r="E13" s="44" t="n">
         <v>3200</v>
       </c>
-      <c r="E13" s="41" t="n">
+      <c r="F13" s="41" t="n">
         <v>3900</v>
       </c>
     </row>
@@ -1080,15 +1180,20 @@
           <t>Ceremonies &amp; Protocol</t>
         </is>
       </c>
-      <c r="C14" s="37" t="inlineStr">
+      <c r="C14" s="80" t="inlineStr">
+        <is>
+          <t>ورشة التشريفات والبروتوكول</t>
+        </is>
+      </c>
+      <c r="D14" s="37" t="inlineStr">
         <is>
           <t>Events &amp; Protocol</t>
         </is>
       </c>
-      <c r="D14" s="38" t="n">
+      <c r="E14" s="38" t="n">
         <v>20001</v>
       </c>
-      <c r="E14" s="41" t="n">
+      <c r="F14" s="41" t="n">
         <v>21750</v>
       </c>
     </row>
@@ -1103,15 +1208,20 @@
           <t>Social Media Coverage</t>
         </is>
       </c>
-      <c r="C15" s="43" t="inlineStr">
+      <c r="C15" s="79" t="inlineStr">
+        <is>
+          <t>ورشة التغطية الإعلامية لوسائل التواصل الاجتماعي</t>
+        </is>
+      </c>
+      <c r="D15" s="43" t="inlineStr">
         <is>
           <t>Social Media &amp; Digital</t>
         </is>
       </c>
-      <c r="D15" s="44" t="n">
+      <c r="E15" s="44" t="n">
         <v>1000</v>
       </c>
-      <c r="E15" s="41" t="n">
+      <c r="F15" s="41" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1126,15 +1236,20 @@
           <t>Photojournalism &amp; Photography</t>
         </is>
       </c>
-      <c r="C16" s="37" t="inlineStr">
+      <c r="C16" s="80" t="inlineStr">
+        <is>
+          <t>ورشة التصوير الصحفي والفوتوغرافي</t>
+        </is>
+      </c>
+      <c r="D16" s="37" t="inlineStr">
         <is>
           <t>Design &amp; Photography</t>
         </is>
       </c>
-      <c r="D16" s="38" t="n">
+      <c r="E16" s="38" t="n">
         <v>648</v>
       </c>
-      <c r="E16" s="41" t="n">
+      <c r="F16" s="41" t="n">
         <v>700</v>
       </c>
     </row>
@@ -1149,15 +1264,20 @@
           <t>Portrait Photography</t>
         </is>
       </c>
-      <c r="C17" s="43" t="inlineStr">
+      <c r="C17" s="79" t="inlineStr">
+        <is>
+          <t>ورشة تصوير البورتريه</t>
+        </is>
+      </c>
+      <c r="D17" s="43" t="inlineStr">
         <is>
           <t>Design &amp; Photography</t>
         </is>
       </c>
-      <c r="D17" s="44" t="n">
+      <c r="E17" s="44" t="n">
         <v>1600</v>
       </c>
-      <c r="E17" s="41" t="n">
+      <c r="F17" s="41" t="n">
         <v>1800</v>
       </c>
     </row>
@@ -1172,15 +1292,20 @@
           <t>Story Telling Workshop</t>
         </is>
       </c>
-      <c r="C18" s="37" t="inlineStr">
+      <c r="C18" s="80" t="inlineStr">
+        <is>
+          <t>Workshop telling Story</t>
+        </is>
+      </c>
+      <c r="D18" s="37" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D18" s="38" t="n">
+      <c r="E18" s="38" t="n">
         <v>9359</v>
       </c>
-      <c r="E18" s="41" t="n">
+      <c r="F18" s="41" t="n">
         <v>10750</v>
       </c>
     </row>
@@ -1195,15 +1320,20 @@
           <t>Media Coverage</t>
         </is>
       </c>
-      <c r="C19" s="43" t="inlineStr">
+      <c r="C19" s="79" t="inlineStr">
+        <is>
+          <t>ورشة التغطيات الإعلامية</t>
+        </is>
+      </c>
+      <c r="D19" s="43" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D19" s="44" t="n">
+      <c r="E19" s="44" t="n">
         <v>15781</v>
       </c>
-      <c r="E19" s="41" t="n">
+      <c r="F19" s="41" t="n">
         <v>17000</v>
       </c>
     </row>
@@ -1218,15 +1348,20 @@
           <t>Law in the Workplace</t>
         </is>
       </c>
-      <c r="C20" s="37" t="inlineStr">
+      <c r="C20" s="80" t="inlineStr">
+        <is>
+          <t>ورشة القانون في مجال العمل</t>
+        </is>
+      </c>
+      <c r="D20" s="37" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D20" s="38" t="n">
+      <c r="E20" s="38" t="n">
         <v>634</v>
       </c>
-      <c r="E20" s="41" t="n">
+      <c r="F20" s="41" t="n">
         <v>650</v>
       </c>
     </row>
@@ -1241,15 +1376,20 @@
           <t>Creative Thinking in the Workplace</t>
         </is>
       </c>
-      <c r="C21" s="43" t="inlineStr">
+      <c r="C21" s="79" t="inlineStr">
+        <is>
+          <t>ورشة التفكير الإبداعي في مجال العمل</t>
+        </is>
+      </c>
+      <c r="D21" s="43" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
       </c>
-      <c r="D21" s="44" t="n">
+      <c r="E21" s="44" t="n">
         <v>6588</v>
       </c>
-      <c r="E21" s="41" t="n">
+      <c r="F21" s="41" t="n">
         <v>7000</v>
       </c>
     </row>
@@ -1264,15 +1404,20 @@
           <t>TV Directing</t>
         </is>
       </c>
-      <c r="C22" s="37" t="inlineStr">
+      <c r="C22" s="80" t="inlineStr">
+        <is>
+          <t>ورشة الإخراج التلفزيوني</t>
+        </is>
+      </c>
+      <c r="D22" s="37" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D22" s="38" t="n">
+      <c r="E22" s="38" t="n">
         <v>4250</v>
       </c>
-      <c r="E22" s="41" t="n">
+      <c r="F22" s="41" t="n">
         <v>4500</v>
       </c>
     </row>
@@ -1287,15 +1432,20 @@
           <t>TV Editing / Montage</t>
         </is>
       </c>
-      <c r="C23" s="43" t="inlineStr">
+      <c r="C23" s="79" t="inlineStr">
+        <is>
+          <t>ورشة المونتاج التلفزيوني</t>
+        </is>
+      </c>
+      <c r="D23" s="43" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D23" s="44" t="n">
+      <c r="E23" s="44" t="n">
         <v>3000</v>
       </c>
-      <c r="E23" s="41" t="n">
+      <c r="F23" s="41" t="n">
         <v>3000</v>
       </c>
     </row>
@@ -1310,15 +1460,20 @@
           <t>Verifying Information on Social Media</t>
         </is>
       </c>
-      <c r="C24" s="37" t="inlineStr">
+      <c r="C24" s="80" t="inlineStr">
+        <is>
+          <t>ورشة التحقق من المعلومات المنشورة على وسائل التواصل الاجتماعي</t>
+        </is>
+      </c>
+      <c r="D24" s="37" t="inlineStr">
         <is>
           <t>Social Media &amp; Digital</t>
         </is>
       </c>
-      <c r="D24" s="38" t="n">
+      <c r="E24" s="38" t="n">
         <v>1800</v>
       </c>
-      <c r="E24" s="41" t="n">
+      <c r="F24" s="41" t="n">
         <v>1900</v>
       </c>
     </row>
@@ -1333,15 +1488,20 @@
           <t>Social Media Graphic Design &amp; Coordination</t>
         </is>
       </c>
-      <c r="C25" s="43" t="inlineStr">
+      <c r="C25" s="79" t="inlineStr">
+        <is>
+          <t>ورشة تنسيق وتصميم الجرافيك لوسائل التواصل الاجتماعي</t>
+        </is>
+      </c>
+      <c r="D25" s="43" t="inlineStr">
         <is>
           <t>Social Media &amp; Digital</t>
         </is>
       </c>
-      <c r="D25" s="44" t="n">
+      <c r="E25" s="44" t="n">
         <v>2150</v>
       </c>
-      <c r="E25" s="41" t="n">
+      <c r="F25" s="41" t="n">
         <v>3300</v>
       </c>
     </row>
@@ -1356,15 +1516,20 @@
           <t>Graphic Design</t>
         </is>
       </c>
-      <c r="C26" s="37" t="inlineStr">
+      <c r="C26" s="80" t="inlineStr">
+        <is>
+          <t>ورشة تصميم الجرافيك</t>
+        </is>
+      </c>
+      <c r="D26" s="37" t="inlineStr">
         <is>
           <t>Design &amp; Photography</t>
         </is>
       </c>
-      <c r="D26" s="38" t="n">
+      <c r="E26" s="38" t="n">
         <v>1550</v>
       </c>
-      <c r="E26" s="41" t="n">
+      <c r="F26" s="41" t="n">
         <v>1600</v>
       </c>
     </row>
@@ -1379,15 +1544,20 @@
           <t>Strategic Communication</t>
         </is>
       </c>
-      <c r="C27" s="43" t="inlineStr">
+      <c r="C27" s="79" t="inlineStr">
+        <is>
+          <t>ورشة الاتصال الاستراتيجي</t>
+        </is>
+      </c>
+      <c r="D27" s="43" t="inlineStr">
         <is>
           <t>Social Media &amp; Digital</t>
         </is>
       </c>
-      <c r="D27" s="44" t="n">
+      <c r="E27" s="44" t="n">
         <v>4600</v>
       </c>
-      <c r="E27" s="41" t="n">
+      <c r="F27" s="41" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -1402,15 +1572,20 @@
           <t>Website Content Management</t>
         </is>
       </c>
-      <c r="C28" s="37" t="inlineStr">
+      <c r="C28" s="80" t="inlineStr">
+        <is>
+          <t>ورشة إدارة محتوى المواقع الإلكترونية</t>
+        </is>
+      </c>
+      <c r="D28" s="37" t="inlineStr">
         <is>
           <t>Technology &amp; Cybersecurity</t>
         </is>
       </c>
-      <c r="D28" s="38" t="n">
+      <c r="E28" s="38" t="n">
         <v>3000</v>
       </c>
-      <c r="E28" s="41" t="n">
+      <c r="F28" s="41" t="n">
         <v>3200</v>
       </c>
     </row>
@@ -1425,15 +1600,20 @@
           <t>Financial Budgets</t>
         </is>
       </c>
-      <c r="C29" s="43" t="inlineStr">
+      <c r="C29" s="79" t="inlineStr">
+        <is>
+          <t>ورشة الموازنات المالية</t>
+        </is>
+      </c>
+      <c r="D29" s="43" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
       </c>
-      <c r="D29" s="44" t="n">
+      <c r="E29" s="44" t="n">
         <v>15793</v>
       </c>
-      <c r="E29" s="41" t="n">
+      <c r="F29" s="41" t="n">
         <v>18250</v>
       </c>
     </row>
@@ -1448,15 +1628,20 @@
           <t>Computer Applications Skills</t>
         </is>
       </c>
-      <c r="C30" s="37" t="inlineStr">
+      <c r="C30" s="80" t="inlineStr">
+        <is>
+          <t>ورشة مهارات استخدام تطبيقات الحاسوب</t>
+        </is>
+      </c>
+      <c r="D30" s="37" t="inlineStr">
         <is>
           <t>Technology &amp; Cybersecurity</t>
         </is>
       </c>
-      <c r="D30" s="38" t="n">
+      <c r="E30" s="38" t="n">
         <v>1675</v>
       </c>
-      <c r="E30" s="41" t="n">
+      <c r="F30" s="41" t="n">
         <v>1800</v>
       </c>
     </row>
@@ -1471,33 +1656,38 @@
           <t>Cybersecurity &amp; Protection from Hacking</t>
         </is>
       </c>
-      <c r="C31" s="43" t="inlineStr">
+      <c r="C31" s="79" t="inlineStr">
+        <is>
+          <t>ورشة الوقاية والحماية من الاختراقات</t>
+        </is>
+      </c>
+      <c r="D31" s="43" t="inlineStr">
         <is>
           <t>Technology &amp; Cybersecurity</t>
         </is>
       </c>
-      <c r="D31" s="44" t="n">
+      <c r="E31" s="44" t="n">
         <v>2810</v>
       </c>
-      <c r="E31" s="41" t="n">
+      <c r="F31" s="41" t="n">
         <v>3100</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="71" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E32" s="72" t="n">
+          <t>TOTAL  |  الإجمالي</t>
+        </is>
+      </c>
+      <c r="F32" s="72" t="n">
         <v>184500</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A32:E32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1509,113 +1699,120 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="27" min="1" max="1"/>
-    <col width="34" customWidth="1" style="27" min="2" max="2"/>
-    <col width="26" customWidth="1" style="27" min="3" max="3"/>
-    <col width="12" customWidth="1" style="27" min="4" max="4"/>
-    <col width="14" customWidth="1" style="27" min="5" max="5"/>
-    <col width="12" customWidth="1" style="27" min="6" max="6"/>
-    <col width="13" customWidth="1" style="27" min="7" max="7"/>
-    <col width="16" customWidth="1" style="27" min="8" max="8"/>
-    <col width="13" customWidth="1" style="27" min="9" max="9"/>
+    <col width="32" customWidth="1" style="27" min="2" max="2"/>
+    <col width="30" customWidth="1" style="27" min="3" max="3"/>
+    <col width="24" customWidth="1" style="27" min="4" max="4"/>
+    <col width="11" customWidth="1" style="27" min="5" max="5"/>
+    <col width="13" customWidth="1" style="27" min="6" max="6"/>
+    <col width="11" customWidth="1" style="27" min="7" max="7"/>
+    <col width="13" customWidth="1" style="27" min="8" max="8"/>
+    <col width="16" customWidth="1" style="27" min="9" max="9"/>
     <col width="13" customWidth="1" style="27" min="10" max="10"/>
-    <col width="34" customWidth="1" style="27" min="11" max="11"/>
+    <col width="13" customWidth="1" style="27" min="11" max="11"/>
+    <col width="32" customWidth="1" style="27" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="28" t="inlineStr">
         <is>
-          <t>SGMB Workshop Pricing — Recommended SGMB Prices vs Competitor Market</t>
+          <t>SGMB Workshop Pricing — Recommended Prices vs Competitor Market  |  تسعير ورش العمل</t>
         </is>
       </c>
     </row>
     <row r="2" ht="58" customHeight="1" s="27">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Positioning: Premium / government-quality — SGMB priced at the upper-mid of the market (above median). Full Course = complete multi-day workshop. One-Day Workshop = condensed single intensive day. Online Class = remote delivery (most accessible). Methodology: Full Course = ~60th percentile of confirmed competitor prices (floored at median +5%, capped at 90th percentile to avoid outliers); One-Day = 50% of Full Course; Online = 40% of Full Course. USD 1=3.67 / EUR 1=4.07 AED. Prices exclude 5% VAT.</t>
+          <t>Positioning: Premium / government-quality — SGMB priced at the upper-mid of the market (above median). Full Course = complete multi-day workshop. One-Day Workshop = condensed single intensive day. Online Class = remote delivery. Methodology: Full Course = ~60th percentile of competitor prices (floored at median +5%, capped at 90th percentile); One-Day = 50% of Full Course; Online = 40%. USD 1=3.67 / EUR 1=4.07 AED. Prices exclude 5% VAT.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="30" t="inlineStr">
         <is>
-          <t>WORKSHOP</t>
-        </is>
-      </c>
-      <c r="B4" s="73" t="n"/>
-      <c r="C4" s="74" t="n"/>
-      <c r="D4" s="31" t="inlineStr">
+          <t>WORKSHOP  |  الورشة</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="n"/>
+      <c r="C4" s="30" t="n"/>
+      <c r="D4" s="30" t="n"/>
+      <c r="E4" s="31" t="inlineStr">
         <is>
           <t>COMPETITOR MARKET (AED)</t>
         </is>
       </c>
-      <c r="E4" s="73" t="n"/>
-      <c r="F4" s="74" t="n"/>
-      <c r="G4" s="30" t="inlineStr">
+      <c r="F4" s="31" t="n"/>
+      <c r="G4" s="31" t="n"/>
+      <c r="H4" s="30" t="inlineStr">
         <is>
           <t>RECOMMENDED SGMB PRICE (AED)</t>
         </is>
       </c>
-      <c r="H4" s="73" t="n"/>
-      <c r="I4" s="74" t="n"/>
-      <c r="J4" s="30" t="inlineStr"/>
-      <c r="K4" s="30" t="inlineStr"/>
+      <c r="I4" s="30" t="n"/>
+      <c r="J4" s="30" t="n"/>
+      <c r="K4" s="81" t="n"/>
+      <c r="L4" s="81" t="n"/>
     </row>
     <row r="5" ht="34" customHeight="1" s="27">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" s="82" t="inlineStr">
         <is>
           <t>SGMB Code</t>
         </is>
       </c>
-      <c r="B5" s="32" t="inlineStr">
+      <c r="B5" s="82" t="inlineStr">
         <is>
           <t>Workshop Name</t>
         </is>
       </c>
-      <c r="C5" s="32" t="inlineStr">
+      <c r="C5" s="83" t="inlineStr">
+        <is>
+          <t>اسم الورشة</t>
+        </is>
+      </c>
+      <c r="D5" s="82" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="E5" s="77" t="inlineStr">
         <is>
           <t>Market Min</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="F5" s="77" t="inlineStr">
         <is>
           <t>Market Median</t>
         </is>
       </c>
-      <c r="F5" s="31" t="inlineStr">
+      <c r="G5" s="77" t="inlineStr">
         <is>
           <t>Market Max</t>
         </is>
       </c>
-      <c r="G5" s="33" t="inlineStr">
+      <c r="H5" s="84" t="inlineStr">
         <is>
           <t>Online Class</t>
         </is>
       </c>
-      <c r="H5" s="34" t="inlineStr">
+      <c r="I5" s="85" t="inlineStr">
         <is>
           <t>One-Day Workshop</t>
         </is>
       </c>
-      <c r="I5" s="35" t="inlineStr">
+      <c r="J5" s="78" t="inlineStr">
         <is>
           <t>Full Course</t>
         </is>
       </c>
-      <c r="J5" s="32" t="inlineStr">
+      <c r="K5" s="82" t="inlineStr">
         <is>
           <t>Full Course Hrs</t>
         </is>
       </c>
-      <c r="K5" s="32" t="inlineStr">
+      <c r="L5" s="82" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1632,33 +1829,38 @@
           <t>Media Communication Fundamentals</t>
         </is>
       </c>
-      <c r="C6" s="37" t="inlineStr">
+      <c r="C6" s="80" t="inlineStr">
+        <is>
+          <t>ورشة أصول التعامل الإعلامي</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D6" s="38" t="n">
+      <c r="E6" s="38" t="n">
         <v>899</v>
       </c>
-      <c r="E6" s="38" t="n">
+      <c r="F6" s="38" t="n">
         <v>10826</v>
       </c>
-      <c r="F6" s="38" t="n">
+      <c r="G6" s="38" t="n">
         <v>18166</v>
       </c>
-      <c r="G6" s="39" t="n">
+      <c r="H6" s="39" t="n">
         <v>5500</v>
       </c>
-      <c r="H6" s="40" t="n">
+      <c r="I6" s="40" t="n">
         <v>7000</v>
       </c>
-      <c r="I6" s="41" t="n">
+      <c r="J6" s="41" t="n">
         <v>13750</v>
       </c>
-      <c r="J6" s="36" t="n">
+      <c r="K6" s="36" t="n">
         <v>21</v>
       </c>
-      <c r="K6" s="37" t="inlineStr"/>
+      <c r="L6" s="37" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="42" t="inlineStr">
@@ -1671,33 +1873,38 @@
           <t>Digital Journalism</t>
         </is>
       </c>
-      <c r="C7" s="43" t="inlineStr">
+      <c r="C7" s="79" t="inlineStr">
+        <is>
+          <t>ورشة الصحافة الرقمية</t>
+        </is>
+      </c>
+      <c r="D7" s="43" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D7" s="44" t="n">
+      <c r="E7" s="44" t="n">
         <v>899</v>
       </c>
-      <c r="E7" s="44" t="n">
+      <c r="F7" s="44" t="n">
         <v>5505</v>
       </c>
-      <c r="F7" s="44" t="n">
+      <c r="G7" s="44" t="n">
         <v>8000</v>
       </c>
-      <c r="G7" s="39" t="n">
+      <c r="H7" s="39" t="n">
         <v>2400</v>
       </c>
-      <c r="H7" s="40" t="n">
+      <c r="I7" s="40" t="n">
         <v>3000</v>
       </c>
-      <c r="I7" s="41" t="n">
+      <c r="J7" s="41" t="n">
         <v>6000</v>
       </c>
-      <c r="J7" s="42" t="n">
+      <c r="K7" s="42" t="n">
         <v>21</v>
       </c>
-      <c r="K7" s="43" t="inlineStr"/>
+      <c r="L7" s="43" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="36" t="inlineStr">
@@ -1710,33 +1917,38 @@
           <t>TV Reporting</t>
         </is>
       </c>
-      <c r="C8" s="37" t="inlineStr">
+      <c r="C8" s="80" t="inlineStr">
+        <is>
+          <t>ورشة التقرير التلفزيوني</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D8" s="38" t="n">
+      <c r="E8" s="38" t="n">
         <v>899</v>
       </c>
-      <c r="E8" s="38" t="n">
+      <c r="F8" s="38" t="n">
         <v>5000</v>
       </c>
-      <c r="F8" s="38" t="n">
+      <c r="G8" s="38" t="n">
         <v>11395</v>
       </c>
-      <c r="G8" s="39" t="n">
+      <c r="H8" s="39" t="n">
         <v>2100</v>
       </c>
-      <c r="H8" s="40" t="n">
+      <c r="I8" s="40" t="n">
         <v>2600</v>
       </c>
-      <c r="I8" s="41" t="n">
+      <c r="J8" s="41" t="n">
         <v>5250</v>
       </c>
-      <c r="J8" s="36" t="n">
+      <c r="K8" s="36" t="n">
         <v>24</v>
       </c>
-      <c r="K8" s="37" t="inlineStr">
+      <c r="L8" s="37" t="inlineStr">
         <is>
           <t>Limited market data.</t>
         </is>
@@ -1753,13 +1965,15 @@
           <t>Job Interview Track</t>
         </is>
       </c>
-      <c r="C9" s="43" t="inlineStr">
+      <c r="C9" s="79" t="inlineStr">
+        <is>
+          <t>ورشة مسار المقابلات الوظيفية</t>
+        </is>
+      </c>
+      <c r="D9" s="43" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
-      </c>
-      <c r="D9" s="44" t="n">
-        <v>6591</v>
       </c>
       <c r="E9" s="44" t="n">
         <v>6591</v>
@@ -1767,19 +1981,22 @@
       <c r="F9" s="44" t="n">
         <v>6591</v>
       </c>
-      <c r="G9" s="39" t="n">
+      <c r="G9" s="44" t="n">
+        <v>6591</v>
+      </c>
+      <c r="H9" s="39" t="n">
         <v>2600</v>
       </c>
-      <c r="H9" s="40" t="n">
+      <c r="I9" s="40" t="n">
         <v>3200</v>
       </c>
-      <c r="I9" s="41" t="n">
+      <c r="J9" s="41" t="n">
         <v>6500</v>
       </c>
-      <c r="J9" s="42" t="n">
+      <c r="K9" s="42" t="n">
         <v>18</v>
       </c>
-      <c r="K9" s="43" t="inlineStr">
+      <c r="L9" s="43" t="inlineStr">
         <is>
           <t>Only 1 confirmed market price.</t>
         </is>
@@ -1796,33 +2013,38 @@
           <t>Art of Management</t>
         </is>
       </c>
-      <c r="C10" s="37" t="inlineStr">
+      <c r="C10" s="80" t="inlineStr">
+        <is>
+          <t>ورشة فن الإدارة</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
       </c>
-      <c r="D10" s="38" t="n">
+      <c r="E10" s="38" t="n">
         <v>9359</v>
       </c>
-      <c r="E10" s="38" t="n">
+      <c r="F10" s="38" t="n">
         <v>13671</v>
       </c>
-      <c r="F10" s="38" t="n">
+      <c r="G10" s="38" t="n">
         <v>17983</v>
       </c>
-      <c r="G10" s="39" t="n">
+      <c r="H10" s="39" t="n">
         <v>5750</v>
       </c>
-      <c r="H10" s="40" t="n">
+      <c r="I10" s="40" t="n">
         <v>7250</v>
       </c>
-      <c r="I10" s="41" t="n">
+      <c r="J10" s="41" t="n">
         <v>14500</v>
       </c>
-      <c r="J10" s="36" t="n">
+      <c r="K10" s="36" t="n">
         <v>24</v>
       </c>
-      <c r="K10" s="37" t="inlineStr"/>
+      <c r="L10" s="37" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="42" t="inlineStr">
@@ -1835,33 +2057,38 @@
           <t>Journalistic Workshop</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="79" t="inlineStr">
+        <is>
+          <t>الورشة الصحفية</t>
+        </is>
+      </c>
+      <c r="D11" s="43" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D11" s="44" t="n">
+      <c r="E11" s="44" t="n">
         <v>899</v>
       </c>
-      <c r="E11" s="44" t="n">
+      <c r="F11" s="44" t="n">
         <v>3745</v>
       </c>
-      <c r="F11" s="44" t="n">
+      <c r="G11" s="44" t="n">
         <v>6591</v>
       </c>
-      <c r="G11" s="39" t="n">
+      <c r="H11" s="39" t="n">
         <v>1700</v>
       </c>
-      <c r="H11" s="40" t="n">
+      <c r="I11" s="40" t="n">
         <v>2200</v>
       </c>
-      <c r="I11" s="41" t="n">
+      <c r="J11" s="41" t="n">
         <v>4300</v>
       </c>
-      <c r="J11" s="42" t="n">
+      <c r="K11" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="K11" s="43" t="inlineStr"/>
+      <c r="L11" s="43" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
@@ -1874,33 +2101,38 @@
           <t>International Forums Organization</t>
         </is>
       </c>
-      <c r="C12" s="37" t="inlineStr">
+      <c r="C12" s="80" t="inlineStr">
+        <is>
+          <t>ورشة تنظيم المنتديات الدولية</t>
+        </is>
+      </c>
+      <c r="D12" s="37" t="inlineStr">
         <is>
           <t>Events &amp; Protocol</t>
         </is>
       </c>
-      <c r="D12" s="38" t="n">
+      <c r="E12" s="38" t="n">
         <v>999</v>
       </c>
-      <c r="E12" s="38" t="n">
+      <c r="F12" s="38" t="n">
         <v>4300</v>
       </c>
-      <c r="F12" s="38" t="n">
+      <c r="G12" s="38" t="n">
         <v>21836</v>
       </c>
-      <c r="G12" s="39" t="n">
+      <c r="H12" s="39" t="n">
         <v>4700</v>
       </c>
-      <c r="H12" s="40" t="n">
+      <c r="I12" s="40" t="n">
         <v>6000</v>
       </c>
-      <c r="I12" s="41" t="n">
+      <c r="J12" s="41" t="n">
         <v>11750</v>
       </c>
-      <c r="J12" s="36" t="n">
+      <c r="K12" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="K12" s="37" t="inlineStr"/>
+      <c r="L12" s="37" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="42" t="inlineStr">
@@ -1913,33 +2145,38 @@
           <t>Official Email Correspondence</t>
         </is>
       </c>
-      <c r="C13" s="43" t="inlineStr">
+      <c r="C13" s="79" t="inlineStr">
+        <is>
+          <t>ورشة المخاطبات الرسمية بالبريد الإلكتروني</t>
+        </is>
+      </c>
+      <c r="D13" s="43" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
       </c>
-      <c r="D13" s="44" t="n">
+      <c r="E13" s="44" t="n">
         <v>999</v>
       </c>
-      <c r="E13" s="44" t="n">
+      <c r="F13" s="44" t="n">
         <v>9359</v>
       </c>
-      <c r="F13" s="44" t="n">
+      <c r="G13" s="44" t="n">
         <v>15781</v>
       </c>
-      <c r="G13" s="39" t="n">
+      <c r="H13" s="39" t="n">
         <v>4300</v>
       </c>
-      <c r="H13" s="40" t="n">
+      <c r="I13" s="40" t="n">
         <v>5500</v>
       </c>
-      <c r="I13" s="41" t="n">
+      <c r="J13" s="41" t="n">
         <v>10750</v>
       </c>
-      <c r="J13" s="42" t="n">
+      <c r="K13" s="42" t="n">
         <v>21</v>
       </c>
-      <c r="K13" s="43" t="inlineStr"/>
+      <c r="L13" s="43" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="36" t="inlineStr">
@@ -1952,33 +2189,38 @@
           <t>Event Management</t>
         </is>
       </c>
-      <c r="C14" s="37" t="inlineStr">
+      <c r="C14" s="80" t="inlineStr">
+        <is>
+          <t>ورشة تنظيم الفعاليات</t>
+        </is>
+      </c>
+      <c r="D14" s="37" t="inlineStr">
         <is>
           <t>Events &amp; Protocol</t>
         </is>
       </c>
-      <c r="D14" s="38" t="n">
+      <c r="E14" s="38" t="n">
         <v>1500</v>
       </c>
-      <c r="E14" s="38" t="n">
+      <c r="F14" s="38" t="n">
         <v>3200</v>
       </c>
-      <c r="F14" s="38" t="n">
+      <c r="G14" s="38" t="n">
         <v>13204</v>
       </c>
-      <c r="G14" s="39" t="n">
+      <c r="H14" s="39" t="n">
         <v>1600</v>
       </c>
-      <c r="H14" s="40" t="n">
+      <c r="I14" s="40" t="n">
         <v>2000</v>
       </c>
-      <c r="I14" s="41" t="n">
+      <c r="J14" s="41" t="n">
         <v>3900</v>
       </c>
-      <c r="J14" s="36" t="n">
+      <c r="K14" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="K14" s="37" t="inlineStr"/>
+      <c r="L14" s="37" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="42" t="inlineStr">
@@ -1991,33 +2233,38 @@
           <t>Ceremonies &amp; Protocol</t>
         </is>
       </c>
-      <c r="C15" s="43" t="inlineStr">
+      <c r="C15" s="79" t="inlineStr">
+        <is>
+          <t>ورشة التشريفات والبروتوكول</t>
+        </is>
+      </c>
+      <c r="D15" s="43" t="inlineStr">
         <is>
           <t>Events &amp; Protocol</t>
         </is>
       </c>
-      <c r="D15" s="44" t="n">
+      <c r="E15" s="44" t="n">
         <v>3500</v>
       </c>
-      <c r="E15" s="44" t="n">
+      <c r="F15" s="44" t="n">
         <v>20001</v>
       </c>
-      <c r="F15" s="44" t="n">
+      <c r="G15" s="44" t="n">
         <v>28906</v>
       </c>
-      <c r="G15" s="39" t="n">
+      <c r="H15" s="39" t="n">
         <v>8750</v>
       </c>
-      <c r="H15" s="40" t="n">
+      <c r="I15" s="40" t="n">
         <v>11000</v>
       </c>
-      <c r="I15" s="41" t="n">
+      <c r="J15" s="41" t="n">
         <v>21750</v>
       </c>
-      <c r="J15" s="42" t="n">
+      <c r="K15" s="42" t="n">
         <v>24</v>
       </c>
-      <c r="K15" s="43" t="inlineStr"/>
+      <c r="L15" s="43" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="36" t="inlineStr">
@@ -2030,33 +2277,38 @@
           <t>Social Media Coverage</t>
         </is>
       </c>
-      <c r="C16" s="37" t="inlineStr">
+      <c r="C16" s="80" t="inlineStr">
+        <is>
+          <t>ورشة التغطية الإعلامية لوسائل التواصل الاجتماعي</t>
+        </is>
+      </c>
+      <c r="D16" s="37" t="inlineStr">
         <is>
           <t>Social Media &amp; Digital</t>
         </is>
       </c>
-      <c r="D16" s="38" t="n">
+      <c r="E16" s="38" t="n">
         <v>441</v>
       </c>
-      <c r="E16" s="38" t="n">
+      <c r="F16" s="38" t="n">
         <v>1000</v>
       </c>
-      <c r="F16" s="38" t="n">
+      <c r="G16" s="38" t="n">
         <v>5000</v>
       </c>
-      <c r="G16" s="39" t="n">
+      <c r="H16" s="39" t="n">
         <v>800</v>
       </c>
-      <c r="H16" s="40" t="n">
+      <c r="I16" s="40" t="n">
         <v>1000</v>
       </c>
-      <c r="I16" s="41" t="n">
+      <c r="J16" s="41" t="n">
         <v>2000</v>
       </c>
-      <c r="J16" s="36" t="n">
+      <c r="K16" s="36" t="n">
         <v>12</v>
       </c>
-      <c r="K16" s="37" t="inlineStr"/>
+      <c r="L16" s="37" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="42" t="inlineStr">
@@ -2069,33 +2321,38 @@
           <t>Photojournalism &amp; Photography</t>
         </is>
       </c>
-      <c r="C17" s="43" t="inlineStr">
+      <c r="C17" s="79" t="inlineStr">
+        <is>
+          <t>ورشة التصوير الصحفي والفوتوغرافي</t>
+        </is>
+      </c>
+      <c r="D17" s="43" t="inlineStr">
         <is>
           <t>Design &amp; Photography</t>
         </is>
       </c>
-      <c r="D17" s="44" t="n">
+      <c r="E17" s="44" t="n">
         <v>350</v>
       </c>
-      <c r="E17" s="44" t="n">
+      <c r="F17" s="44" t="n">
         <v>648</v>
       </c>
-      <c r="F17" s="44" t="n">
+      <c r="G17" s="44" t="n">
         <v>2800</v>
       </c>
-      <c r="G17" s="39" t="n">
+      <c r="H17" s="39" t="n">
         <v>275</v>
       </c>
-      <c r="H17" s="40" t="n">
+      <c r="I17" s="40" t="n">
         <v>350</v>
       </c>
-      <c r="I17" s="41" t="n">
+      <c r="J17" s="41" t="n">
         <v>700</v>
       </c>
-      <c r="J17" s="42" t="n">
+      <c r="K17" s="42" t="n">
         <v>12</v>
       </c>
-      <c r="K17" s="43" t="inlineStr"/>
+      <c r="L17" s="43" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="36" t="inlineStr">
@@ -2108,33 +2365,38 @@
           <t>Portrait Photography</t>
         </is>
       </c>
-      <c r="C18" s="37" t="inlineStr">
+      <c r="C18" s="80" t="inlineStr">
+        <is>
+          <t>ورشة تصوير البورتريه</t>
+        </is>
+      </c>
+      <c r="D18" s="37" t="inlineStr">
         <is>
           <t>Design &amp; Photography</t>
         </is>
       </c>
-      <c r="D18" s="38" t="n">
+      <c r="E18" s="38" t="n">
         <v>595</v>
       </c>
-      <c r="E18" s="38" t="n">
+      <c r="F18" s="38" t="n">
         <v>1600</v>
       </c>
-      <c r="F18" s="38" t="n">
+      <c r="G18" s="38" t="n">
         <v>1900</v>
       </c>
-      <c r="G18" s="39" t="n">
+      <c r="H18" s="39" t="n">
         <v>700</v>
       </c>
-      <c r="H18" s="40" t="n">
+      <c r="I18" s="40" t="n">
         <v>900</v>
       </c>
-      <c r="I18" s="41" t="n">
+      <c r="J18" s="41" t="n">
         <v>1800</v>
       </c>
-      <c r="J18" s="36" t="n">
+      <c r="K18" s="36" t="n">
         <v>12</v>
       </c>
-      <c r="K18" s="37" t="inlineStr"/>
+      <c r="L18" s="37" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="42" t="inlineStr">
@@ -2147,33 +2409,38 @@
           <t>Story Telling Workshop</t>
         </is>
       </c>
-      <c r="C19" s="43" t="inlineStr">
+      <c r="C19" s="79" t="inlineStr">
+        <is>
+          <t>Workshop telling Story</t>
+        </is>
+      </c>
+      <c r="D19" s="43" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D19" s="44" t="n">
+      <c r="E19" s="44" t="n">
         <v>180</v>
       </c>
-      <c r="E19" s="44" t="n">
+      <c r="F19" s="44" t="n">
         <v>9359</v>
       </c>
-      <c r="F19" s="44" t="n">
+      <c r="G19" s="44" t="n">
         <v>15781</v>
       </c>
-      <c r="G19" s="39" t="n">
+      <c r="H19" s="39" t="n">
         <v>4300</v>
       </c>
-      <c r="H19" s="40" t="n">
+      <c r="I19" s="40" t="n">
         <v>5500</v>
       </c>
-      <c r="I19" s="41" t="n">
+      <c r="J19" s="41" t="n">
         <v>10750</v>
       </c>
-      <c r="J19" s="42" t="n">
+      <c r="K19" s="42" t="n">
         <v>21</v>
       </c>
-      <c r="K19" s="43" t="inlineStr"/>
+      <c r="L19" s="43" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="36" t="inlineStr">
@@ -2186,33 +2453,38 @@
           <t>Media Coverage</t>
         </is>
       </c>
-      <c r="C20" s="37" t="inlineStr">
+      <c r="C20" s="80" t="inlineStr">
+        <is>
+          <t>ورشة التغطيات الإعلامية</t>
+        </is>
+      </c>
+      <c r="D20" s="37" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D20" s="38" t="n">
+      <c r="E20" s="38" t="n">
         <v>899</v>
       </c>
-      <c r="E20" s="38" t="n">
+      <c r="F20" s="38" t="n">
         <v>15781</v>
       </c>
-      <c r="F20" s="38" t="n">
+      <c r="G20" s="38" t="n">
         <v>21837</v>
       </c>
-      <c r="G20" s="39" t="n">
+      <c r="H20" s="39" t="n">
         <v>6750</v>
       </c>
-      <c r="H20" s="40" t="n">
+      <c r="I20" s="40" t="n">
         <v>8500</v>
       </c>
-      <c r="I20" s="41" t="n">
+      <c r="J20" s="41" t="n">
         <v>17000</v>
       </c>
-      <c r="J20" s="36" t="n">
+      <c r="K20" s="36" t="n">
         <v>24</v>
       </c>
-      <c r="K20" s="37" t="inlineStr"/>
+      <c r="L20" s="37" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="42" t="inlineStr">
@@ -2225,33 +2497,38 @@
           <t>Law in the Workplace</t>
         </is>
       </c>
-      <c r="C21" s="43" t="inlineStr">
+      <c r="C21" s="79" t="inlineStr">
+        <is>
+          <t>ورشة القانون في مجال العمل</t>
+        </is>
+      </c>
+      <c r="D21" s="43" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D21" s="44" t="n">
+      <c r="E21" s="44" t="n">
         <v>570</v>
       </c>
-      <c r="E21" s="44" t="n">
+      <c r="F21" s="44" t="n">
         <v>634</v>
       </c>
-      <c r="F21" s="44" t="n">
+      <c r="G21" s="44" t="n">
         <v>1500</v>
       </c>
-      <c r="G21" s="39" t="n">
+      <c r="H21" s="39" t="n">
         <v>250</v>
       </c>
-      <c r="H21" s="40" t="n">
+      <c r="I21" s="40" t="n">
         <v>325</v>
       </c>
-      <c r="I21" s="41" t="n">
+      <c r="J21" s="41" t="n">
         <v>650</v>
       </c>
-      <c r="J21" s="42" t="n">
+      <c r="K21" s="42" t="n">
         <v>12</v>
       </c>
-      <c r="K21" s="43" t="inlineStr"/>
+      <c r="L21" s="43" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="36" t="inlineStr">
@@ -2264,33 +2541,38 @@
           <t>Creative Thinking in the Workplace</t>
         </is>
       </c>
-      <c r="C22" s="37" t="inlineStr">
+      <c r="C22" s="80" t="inlineStr">
+        <is>
+          <t>ورشة التفكير الإبداعي في مجال العمل</t>
+        </is>
+      </c>
+      <c r="D22" s="37" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
       </c>
-      <c r="D22" s="38" t="n">
+      <c r="E22" s="38" t="n">
         <v>4300</v>
       </c>
-      <c r="E22" s="38" t="n">
+      <c r="F22" s="38" t="n">
         <v>6588</v>
       </c>
-      <c r="F22" s="38" t="n">
+      <c r="G22" s="38" t="n">
         <v>17983</v>
       </c>
-      <c r="G22" s="39" t="n">
+      <c r="H22" s="39" t="n">
         <v>2800</v>
       </c>
-      <c r="H22" s="40" t="n">
+      <c r="I22" s="40" t="n">
         <v>3500</v>
       </c>
-      <c r="I22" s="41" t="n">
+      <c r="J22" s="41" t="n">
         <v>7000</v>
       </c>
-      <c r="J22" s="36" t="n">
+      <c r="K22" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="K22" s="37" t="inlineStr"/>
+      <c r="L22" s="37" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="42" t="inlineStr">
@@ -2303,33 +2585,38 @@
           <t>TV Directing</t>
         </is>
       </c>
-      <c r="C23" s="43" t="inlineStr">
+      <c r="C23" s="79" t="inlineStr">
+        <is>
+          <t>ورشة الإخراج التلفزيوني</t>
+        </is>
+      </c>
+      <c r="D23" s="43" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
       </c>
-      <c r="D23" s="44" t="n">
+      <c r="E23" s="44" t="n">
         <v>3000</v>
       </c>
-      <c r="E23" s="44" t="n">
+      <c r="F23" s="44" t="n">
         <v>4250</v>
       </c>
-      <c r="F23" s="44" t="n">
+      <c r="G23" s="44" t="n">
         <v>5500</v>
       </c>
-      <c r="G23" s="39" t="n">
+      <c r="H23" s="39" t="n">
         <v>1800</v>
       </c>
-      <c r="H23" s="40" t="n">
+      <c r="I23" s="40" t="n">
         <v>2200</v>
       </c>
-      <c r="I23" s="41" t="n">
+      <c r="J23" s="41" t="n">
         <v>4500</v>
       </c>
-      <c r="J23" s="42" t="n">
+      <c r="K23" s="42" t="n">
         <v>24</v>
       </c>
-      <c r="K23" s="43" t="inlineStr"/>
+      <c r="L23" s="43" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="36" t="inlineStr">
@@ -2342,13 +2629,15 @@
           <t>TV Editing / Montage</t>
         </is>
       </c>
-      <c r="C24" s="37" t="inlineStr">
+      <c r="C24" s="80" t="inlineStr">
+        <is>
+          <t>ورشة المونتاج التلفزيوني</t>
+        </is>
+      </c>
+      <c r="D24" s="37" t="inlineStr">
         <is>
           <t>Media &amp; Journalism</t>
         </is>
-      </c>
-      <c r="D24" s="38" t="n">
-        <v>3000</v>
       </c>
       <c r="E24" s="38" t="n">
         <v>3000</v>
@@ -2356,19 +2645,22 @@
       <c r="F24" s="38" t="n">
         <v>3000</v>
       </c>
-      <c r="G24" s="39" t="n">
+      <c r="G24" s="38" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H24" s="39" t="n">
         <v>1200</v>
       </c>
-      <c r="H24" s="40" t="n">
+      <c r="I24" s="40" t="n">
         <v>1500</v>
       </c>
-      <c r="I24" s="41" t="n">
+      <c r="J24" s="41" t="n">
         <v>3000</v>
       </c>
-      <c r="J24" s="36" t="n">
+      <c r="K24" s="36" t="n">
         <v>18</v>
       </c>
-      <c r="K24" s="37" t="inlineStr">
+      <c r="L24" s="37" t="inlineStr">
         <is>
           <t>Only 1 confirmed price; often bundled with TV Directing (W18).</t>
         </is>
@@ -2385,33 +2677,38 @@
           <t>Verifying Information on Social Media</t>
         </is>
       </c>
-      <c r="C25" s="43" t="inlineStr">
+      <c r="C25" s="79" t="inlineStr">
+        <is>
+          <t>ورشة التحقق من المعلومات المنشورة على وسائل التواصل الاجتماعي</t>
+        </is>
+      </c>
+      <c r="D25" s="43" t="inlineStr">
         <is>
           <t>Social Media &amp; Digital</t>
         </is>
       </c>
-      <c r="D25" s="44" t="n">
+      <c r="E25" s="44" t="n">
         <v>500</v>
       </c>
-      <c r="E25" s="44" t="n">
+      <c r="F25" s="44" t="n">
         <v>1800</v>
       </c>
-      <c r="F25" s="44" t="n">
+      <c r="G25" s="44" t="n">
         <v>4753</v>
       </c>
-      <c r="G25" s="39" t="n">
+      <c r="H25" s="39" t="n">
         <v>750</v>
       </c>
-      <c r="H25" s="40" t="n">
+      <c r="I25" s="40" t="n">
         <v>950</v>
       </c>
-      <c r="I25" s="41" t="n">
+      <c r="J25" s="41" t="n">
         <v>1900</v>
       </c>
-      <c r="J25" s="42" t="n">
+      <c r="K25" s="42" t="n">
         <v>21</v>
       </c>
-      <c r="K25" s="43" t="inlineStr">
+      <c r="L25" s="43" t="inlineStr">
         <is>
           <t>Near-unique offering — little direct competition.</t>
         </is>
@@ -2428,33 +2725,38 @@
           <t>Social Media Graphic Design &amp; Coordination</t>
         </is>
       </c>
-      <c r="C26" s="37" t="inlineStr">
+      <c r="C26" s="80" t="inlineStr">
+        <is>
+          <t>ورشة تنسيق وتصميم الجرافيك لوسائل التواصل الاجتماعي</t>
+        </is>
+      </c>
+      <c r="D26" s="37" t="inlineStr">
         <is>
           <t>Social Media &amp; Digital</t>
         </is>
       </c>
-      <c r="D26" s="38" t="n">
+      <c r="E26" s="38" t="n">
         <v>1500</v>
       </c>
-      <c r="E26" s="38" t="n">
+      <c r="F26" s="38" t="n">
         <v>2150</v>
       </c>
-      <c r="F26" s="38" t="n">
+      <c r="G26" s="38" t="n">
         <v>16148</v>
       </c>
-      <c r="G26" s="39" t="n">
+      <c r="H26" s="39" t="n">
         <v>1300</v>
       </c>
-      <c r="H26" s="40" t="n">
+      <c r="I26" s="40" t="n">
         <v>1600</v>
       </c>
-      <c r="I26" s="41" t="n">
+      <c r="J26" s="41" t="n">
         <v>3300</v>
       </c>
-      <c r="J26" s="36" t="n">
+      <c r="K26" s="36" t="n">
         <v>24</v>
       </c>
-      <c r="K26" s="37" t="inlineStr"/>
+      <c r="L26" s="37" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="42" t="inlineStr">
@@ -2467,33 +2769,38 @@
           <t>Graphic Design</t>
         </is>
       </c>
-      <c r="C27" s="43" t="inlineStr">
+      <c r="C27" s="79" t="inlineStr">
+        <is>
+          <t>ورشة تصميم الجرافيك</t>
+        </is>
+      </c>
+      <c r="D27" s="43" t="inlineStr">
         <is>
           <t>Design &amp; Photography</t>
         </is>
       </c>
-      <c r="D27" s="44" t="n">
+      <c r="E27" s="44" t="n">
         <v>1200</v>
       </c>
-      <c r="E27" s="44" t="n">
+      <c r="F27" s="44" t="n">
         <v>1550</v>
       </c>
-      <c r="F27" s="44" t="n">
+      <c r="G27" s="44" t="n">
         <v>9000</v>
       </c>
-      <c r="G27" s="39" t="n">
+      <c r="H27" s="39" t="n">
         <v>650</v>
       </c>
-      <c r="H27" s="40" t="n">
+      <c r="I27" s="40" t="n">
         <v>800</v>
       </c>
-      <c r="I27" s="41" t="n">
+      <c r="J27" s="41" t="n">
         <v>1600</v>
       </c>
-      <c r="J27" s="42" t="n">
+      <c r="K27" s="42" t="n">
         <v>24</v>
       </c>
-      <c r="K27" s="43" t="inlineStr"/>
+      <c r="L27" s="43" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="36" t="inlineStr">
@@ -2506,33 +2813,38 @@
           <t>Strategic Communication</t>
         </is>
       </c>
-      <c r="C28" s="37" t="inlineStr">
+      <c r="C28" s="80" t="inlineStr">
+        <is>
+          <t>ورشة الاتصال الاستراتيجي</t>
+        </is>
+      </c>
+      <c r="D28" s="37" t="inlineStr">
         <is>
           <t>Social Media &amp; Digital</t>
         </is>
       </c>
-      <c r="D28" s="38" t="n">
+      <c r="E28" s="38" t="n">
         <v>3000</v>
       </c>
-      <c r="E28" s="38" t="n">
+      <c r="F28" s="38" t="n">
         <v>4600</v>
       </c>
-      <c r="F28" s="38" t="n">
+      <c r="G28" s="38" t="n">
         <v>21837</v>
       </c>
-      <c r="G28" s="39" t="n">
+      <c r="H28" s="39" t="n">
         <v>2200</v>
       </c>
-      <c r="H28" s="40" t="n">
+      <c r="I28" s="40" t="n">
         <v>2800</v>
       </c>
-      <c r="I28" s="41" t="n">
+      <c r="J28" s="41" t="n">
         <v>5500</v>
       </c>
-      <c r="J28" s="36" t="n">
+      <c r="K28" s="36" t="n">
         <v>21</v>
       </c>
-      <c r="K28" s="37" t="inlineStr"/>
+      <c r="L28" s="37" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="42" t="inlineStr">
@@ -2545,33 +2857,38 @@
           <t>Website Content Management</t>
         </is>
       </c>
-      <c r="C29" s="43" t="inlineStr">
+      <c r="C29" s="79" t="inlineStr">
+        <is>
+          <t>ورشة إدارة محتوى المواقع الإلكترونية</t>
+        </is>
+      </c>
+      <c r="D29" s="43" t="inlineStr">
         <is>
           <t>Technology &amp; Cybersecurity</t>
         </is>
       </c>
-      <c r="D29" s="44" t="n">
+      <c r="E29" s="44" t="n">
         <v>1000</v>
       </c>
-      <c r="E29" s="44" t="n">
+      <c r="F29" s="44" t="n">
         <v>3000</v>
       </c>
-      <c r="F29" s="44" t="n">
+      <c r="G29" s="44" t="n">
         <v>3650</v>
       </c>
-      <c r="G29" s="39" t="n">
+      <c r="H29" s="39" t="n">
         <v>1300</v>
       </c>
-      <c r="H29" s="40" t="n">
+      <c r="I29" s="40" t="n">
         <v>1600</v>
       </c>
-      <c r="I29" s="41" t="n">
+      <c r="J29" s="41" t="n">
         <v>3200</v>
       </c>
-      <c r="J29" s="42" t="n">
+      <c r="K29" s="42" t="n">
         <v>18</v>
       </c>
-      <c r="K29" s="43" t="inlineStr">
+      <c r="L29" s="43" t="inlineStr">
         <is>
           <t>Commoditized (CMS) — kept competitive.</t>
         </is>
@@ -2588,33 +2905,38 @@
           <t>Financial Budgets</t>
         </is>
       </c>
-      <c r="C30" s="37" t="inlineStr">
+      <c r="C30" s="80" t="inlineStr">
+        <is>
+          <t>ورشة الموازنات المالية</t>
+        </is>
+      </c>
+      <c r="D30" s="37" t="inlineStr">
         <is>
           <t>Management &amp; Professional</t>
         </is>
       </c>
-      <c r="D30" s="38" t="n">
+      <c r="E30" s="38" t="n">
         <v>1500</v>
       </c>
-      <c r="E30" s="38" t="n">
+      <c r="F30" s="38" t="n">
         <v>15793</v>
       </c>
-      <c r="F30" s="38" t="n">
+      <c r="G30" s="38" t="n">
         <v>21837</v>
       </c>
-      <c r="G30" s="39" t="n">
+      <c r="H30" s="39" t="n">
         <v>7250</v>
       </c>
-      <c r="H30" s="40" t="n">
+      <c r="I30" s="40" t="n">
         <v>9000</v>
       </c>
-      <c r="I30" s="41" t="n">
+      <c r="J30" s="41" t="n">
         <v>18250</v>
       </c>
-      <c r="J30" s="36" t="n">
+      <c r="K30" s="36" t="n">
         <v>24</v>
       </c>
-      <c r="K30" s="37" t="inlineStr"/>
+      <c r="L30" s="37" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="42" t="inlineStr">
@@ -2627,33 +2949,38 @@
           <t>Computer Applications Skills</t>
         </is>
       </c>
-      <c r="C31" s="43" t="inlineStr">
+      <c r="C31" s="79" t="inlineStr">
+        <is>
+          <t>ورشة مهارات استخدام تطبيقات الحاسوب</t>
+        </is>
+      </c>
+      <c r="D31" s="43" t="inlineStr">
         <is>
           <t>Technology &amp; Cybersecurity</t>
         </is>
       </c>
-      <c r="D31" s="44" t="n">
+      <c r="E31" s="44" t="n">
         <v>180</v>
       </c>
-      <c r="E31" s="44" t="n">
+      <c r="F31" s="44" t="n">
         <v>1675</v>
       </c>
-      <c r="F31" s="44" t="n">
+      <c r="G31" s="44" t="n">
         <v>2500</v>
       </c>
-      <c r="G31" s="39" t="n">
+      <c r="H31" s="39" t="n">
         <v>700</v>
       </c>
-      <c r="H31" s="40" t="n">
+      <c r="I31" s="40" t="n">
         <v>900</v>
       </c>
-      <c r="I31" s="41" t="n">
+      <c r="J31" s="41" t="n">
         <v>1800</v>
       </c>
-      <c r="J31" s="42" t="n">
+      <c r="K31" s="42" t="n">
         <v>24</v>
       </c>
-      <c r="K31" s="43" t="inlineStr">
+      <c r="L31" s="43" t="inlineStr">
         <is>
           <t>Commoditized (MS Office) — kept competitive.</t>
         </is>
@@ -2670,43 +2997,46 @@
           <t>Cybersecurity &amp; Protection from Hacking</t>
         </is>
       </c>
-      <c r="C32" s="37" t="inlineStr">
+      <c r="C32" s="80" t="inlineStr">
+        <is>
+          <t>ورشة الوقاية والحماية من الاختراقات</t>
+        </is>
+      </c>
+      <c r="D32" s="37" t="inlineStr">
         <is>
           <t>Technology &amp; Cybersecurity</t>
         </is>
       </c>
-      <c r="D32" s="38" t="n">
+      <c r="E32" s="38" t="n">
         <v>100</v>
       </c>
-      <c r="E32" s="38" t="n">
+      <c r="F32" s="38" t="n">
         <v>2810</v>
       </c>
-      <c r="F32" s="38" t="n">
+      <c r="G32" s="38" t="n">
         <v>6288</v>
       </c>
-      <c r="G32" s="39" t="n">
+      <c r="H32" s="39" t="n">
         <v>1200</v>
       </c>
-      <c r="H32" s="40" t="n">
+      <c r="I32" s="40" t="n">
         <v>1600</v>
       </c>
-      <c r="I32" s="41" t="n">
+      <c r="J32" s="41" t="n">
         <v>3100</v>
       </c>
-      <c r="J32" s="36" t="n">
+      <c r="K32" s="36" t="n">
         <v>12</v>
       </c>
-      <c r="K32" s="37" t="inlineStr"/>
+      <c r="L32" s="37" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="J4"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="K4"/>
+  <mergeCells count="5">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="A2:M2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Make pricing sheets fully bilingual (headers + categories)
Translate all column headers, group banners, and category names into
Arabic alongside English on both pricing sheets, so the deliverable is
fully bilingual (English / العربية).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjvYXygDKkAN1X1SuAqsBh
</commit_message>
<xml_diff>
--- a/SGMB_Pricing_With_Recommendations.xlsx
+++ b/SGMB_Pricing_With_Recommendations.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -122,6 +122,23 @@
     </font>
     <font>
       <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="23">
@@ -340,7 +357,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -587,6 +604,33 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -885,35 +929,41 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" s="27">
-      <c r="A4" s="75" t="inlineStr">
-        <is>
-          <t>SGMB Code</t>
-        </is>
-      </c>
-      <c r="B4" s="75" t="inlineStr">
-        <is>
-          <t>Workshop Name</t>
+    <row r="4" ht="42" customHeight="1" s="27">
+      <c r="A4" s="76" t="inlineStr">
+        <is>
+          <t>SGMB Code
+رمز الورشة</t>
+        </is>
+      </c>
+      <c r="B4" s="76" t="inlineStr">
+        <is>
+          <t>Workshop Name
+اسم الورشة (إنجليزي)</t>
         </is>
       </c>
       <c r="C4" s="76" t="inlineStr">
         <is>
-          <t>اسم الورشة</t>
-        </is>
-      </c>
-      <c r="D4" s="75" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E4" s="77" t="inlineStr">
-        <is>
-          <t>Market Median (AED)</t>
-        </is>
-      </c>
-      <c r="F4" s="78" t="inlineStr">
-        <is>
-          <t>Recommended Price (AED)</t>
+          <t>اسم الورشة
+Workshop (Arabic)</t>
+        </is>
+      </c>
+      <c r="D4" s="76" t="inlineStr">
+        <is>
+          <t>Category
+الفئة</t>
+        </is>
+      </c>
+      <c r="E4" s="86" t="inlineStr">
+        <is>
+          <t>Market Median (AED)
+متوسط السوق (درهم)</t>
+        </is>
+      </c>
+      <c r="F4" s="87" t="inlineStr">
+        <is>
+          <t>Recommended Price (AED)
+السعر الموصى به (درهم)</t>
         </is>
       </c>
     </row>
@@ -933,9 +983,10 @@
           <t>ورشة أصول التعامل الإعلامي</t>
         </is>
       </c>
-      <c r="D5" s="43" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D5" s="88" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E5" s="44" t="n">
@@ -961,9 +1012,10 @@
           <t>ورشة الصحافة الرقمية</t>
         </is>
       </c>
-      <c r="D6" s="37" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D6" s="89" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E6" s="38" t="n">
@@ -989,9 +1041,10 @@
           <t>ورشة التقرير التلفزيوني</t>
         </is>
       </c>
-      <c r="D7" s="43" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D7" s="88" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E7" s="44" t="n">
@@ -1017,9 +1070,10 @@
           <t>ورشة مسار المقابلات الوظيفية</t>
         </is>
       </c>
-      <c r="D8" s="37" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D8" s="89" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E8" s="38" t="n">
@@ -1045,9 +1099,10 @@
           <t>ورشة فن الإدارة</t>
         </is>
       </c>
-      <c r="D9" s="43" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D9" s="88" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E9" s="44" t="n">
@@ -1073,9 +1128,10 @@
           <t>الورشة الصحفية</t>
         </is>
       </c>
-      <c r="D10" s="37" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D10" s="89" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E10" s="38" t="n">
@@ -1101,9 +1157,10 @@
           <t>ورشة تنظيم المنتديات الدولية</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
-        <is>
-          <t>Events &amp; Protocol</t>
+      <c r="D11" s="88" t="inlineStr">
+        <is>
+          <t>Events &amp; Protocol
+الفعاليات والبروتوكول</t>
         </is>
       </c>
       <c r="E11" s="44" t="n">
@@ -1129,9 +1186,10 @@
           <t>ورشة المخاطبات الرسمية بالبريد الإلكتروني</t>
         </is>
       </c>
-      <c r="D12" s="37" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D12" s="89" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E12" s="38" t="n">
@@ -1157,9 +1215,10 @@
           <t>ورشة تنظيم الفعاليات</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
-        <is>
-          <t>Events &amp; Protocol</t>
+      <c r="D13" s="88" t="inlineStr">
+        <is>
+          <t>Events &amp; Protocol
+الفعاليات والبروتوكول</t>
         </is>
       </c>
       <c r="E13" s="44" t="n">
@@ -1185,9 +1244,10 @@
           <t>ورشة التشريفات والبروتوكول</t>
         </is>
       </c>
-      <c r="D14" s="37" t="inlineStr">
-        <is>
-          <t>Events &amp; Protocol</t>
+      <c r="D14" s="89" t="inlineStr">
+        <is>
+          <t>Events &amp; Protocol
+الفعاليات والبروتوكول</t>
         </is>
       </c>
       <c r="E14" s="38" t="n">
@@ -1213,9 +1273,10 @@
           <t>ورشة التغطية الإعلامية لوسائل التواصل الاجتماعي</t>
         </is>
       </c>
-      <c r="D15" s="43" t="inlineStr">
-        <is>
-          <t>Social Media &amp; Digital</t>
+      <c r="D15" s="88" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital
+التواصل الاجتماعي والرقمي</t>
         </is>
       </c>
       <c r="E15" s="44" t="n">
@@ -1241,9 +1302,10 @@
           <t>ورشة التصوير الصحفي والفوتوغرافي</t>
         </is>
       </c>
-      <c r="D16" s="37" t="inlineStr">
-        <is>
-          <t>Design &amp; Photography</t>
+      <c r="D16" s="89" t="inlineStr">
+        <is>
+          <t>Design &amp; Photography
+التصميم والتصوير</t>
         </is>
       </c>
       <c r="E16" s="38" t="n">
@@ -1269,9 +1331,10 @@
           <t>ورشة تصوير البورتريه</t>
         </is>
       </c>
-      <c r="D17" s="43" t="inlineStr">
-        <is>
-          <t>Design &amp; Photography</t>
+      <c r="D17" s="88" t="inlineStr">
+        <is>
+          <t>Design &amp; Photography
+التصميم والتصوير</t>
         </is>
       </c>
       <c r="E17" s="44" t="n">
@@ -1297,9 +1360,10 @@
           <t>Workshop telling Story</t>
         </is>
       </c>
-      <c r="D18" s="37" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D18" s="89" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E18" s="38" t="n">
@@ -1325,9 +1389,10 @@
           <t>ورشة التغطيات الإعلامية</t>
         </is>
       </c>
-      <c r="D19" s="43" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D19" s="88" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E19" s="44" t="n">
@@ -1353,9 +1418,10 @@
           <t>ورشة القانون في مجال العمل</t>
         </is>
       </c>
-      <c r="D20" s="37" t="inlineStr">
-        <is>
-          <t>Legal</t>
+      <c r="D20" s="89" t="inlineStr">
+        <is>
+          <t>Legal
+القانون</t>
         </is>
       </c>
       <c r="E20" s="38" t="n">
@@ -1381,9 +1447,10 @@
           <t>ورشة التفكير الإبداعي في مجال العمل</t>
         </is>
       </c>
-      <c r="D21" s="43" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D21" s="88" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E21" s="44" t="n">
@@ -1409,9 +1476,10 @@
           <t>ورشة الإخراج التلفزيوني</t>
         </is>
       </c>
-      <c r="D22" s="37" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D22" s="89" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E22" s="38" t="n">
@@ -1437,9 +1505,10 @@
           <t>ورشة المونتاج التلفزيوني</t>
         </is>
       </c>
-      <c r="D23" s="43" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D23" s="88" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E23" s="44" t="n">
@@ -1465,9 +1534,10 @@
           <t>ورشة التحقق من المعلومات المنشورة على وسائل التواصل الاجتماعي</t>
         </is>
       </c>
-      <c r="D24" s="37" t="inlineStr">
-        <is>
-          <t>Social Media &amp; Digital</t>
+      <c r="D24" s="89" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital
+التواصل الاجتماعي والرقمي</t>
         </is>
       </c>
       <c r="E24" s="38" t="n">
@@ -1493,9 +1563,10 @@
           <t>ورشة تنسيق وتصميم الجرافيك لوسائل التواصل الاجتماعي</t>
         </is>
       </c>
-      <c r="D25" s="43" t="inlineStr">
-        <is>
-          <t>Social Media &amp; Digital</t>
+      <c r="D25" s="88" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital
+التواصل الاجتماعي والرقمي</t>
         </is>
       </c>
       <c r="E25" s="44" t="n">
@@ -1521,9 +1592,10 @@
           <t>ورشة تصميم الجرافيك</t>
         </is>
       </c>
-      <c r="D26" s="37" t="inlineStr">
-        <is>
-          <t>Design &amp; Photography</t>
+      <c r="D26" s="89" t="inlineStr">
+        <is>
+          <t>Design &amp; Photography
+التصميم والتصوير</t>
         </is>
       </c>
       <c r="E26" s="38" t="n">
@@ -1549,9 +1621,10 @@
           <t>ورشة الاتصال الاستراتيجي</t>
         </is>
       </c>
-      <c r="D27" s="43" t="inlineStr">
-        <is>
-          <t>Social Media &amp; Digital</t>
+      <c r="D27" s="88" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital
+التواصل الاجتماعي والرقمي</t>
         </is>
       </c>
       <c r="E27" s="44" t="n">
@@ -1577,9 +1650,10 @@
           <t>ورشة إدارة محتوى المواقع الإلكترونية</t>
         </is>
       </c>
-      <c r="D28" s="37" t="inlineStr">
-        <is>
-          <t>Technology &amp; Cybersecurity</t>
+      <c r="D28" s="89" t="inlineStr">
+        <is>
+          <t>Technology &amp; Cybersecurity
+التقنية والأمن السيبراني</t>
         </is>
       </c>
       <c r="E28" s="38" t="n">
@@ -1605,9 +1679,10 @@
           <t>ورشة الموازنات المالية</t>
         </is>
       </c>
-      <c r="D29" s="43" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D29" s="88" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E29" s="44" t="n">
@@ -1633,9 +1708,10 @@
           <t>ورشة مهارات استخدام تطبيقات الحاسوب</t>
         </is>
       </c>
-      <c r="D30" s="37" t="inlineStr">
-        <is>
-          <t>Technology &amp; Cybersecurity</t>
+      <c r="D30" s="89" t="inlineStr">
+        <is>
+          <t>Technology &amp; Cybersecurity
+التقنية والأمن السيبراني</t>
         </is>
       </c>
       <c r="E30" s="38" t="n">
@@ -1661,9 +1737,10 @@
           <t>ورشة الوقاية والحماية من الاختراقات</t>
         </is>
       </c>
-      <c r="D31" s="43" t="inlineStr">
-        <is>
-          <t>Technology &amp; Cybersecurity</t>
+      <c r="D31" s="88" t="inlineStr">
+        <is>
+          <t>Technology &amp; Cybersecurity
+التقنية والأمن السيبراني</t>
         </is>
       </c>
       <c r="E31" s="44" t="n">
@@ -1741,14 +1818,14 @@
       <c r="D4" s="30" t="n"/>
       <c r="E4" s="31" t="inlineStr">
         <is>
-          <t>COMPETITOR MARKET (AED)</t>
+          <t>COMPETITOR MARKET (AED)  |  سوق المنافسين (درهم)</t>
         </is>
       </c>
       <c r="F4" s="31" t="n"/>
       <c r="G4" s="31" t="n"/>
       <c r="H4" s="30" t="inlineStr">
         <is>
-          <t>RECOMMENDED SGMB PRICE (AED)</t>
+          <t>RECOMMENDED SGMB PRICE (AED)  |  السعر الموصى به (درهم)</t>
         </is>
       </c>
       <c r="I4" s="30" t="n"/>
@@ -1756,65 +1833,77 @@
       <c r="K4" s="81" t="n"/>
       <c r="L4" s="81" t="n"/>
     </row>
-    <row r="5" ht="34" customHeight="1" s="27">
-      <c r="A5" s="82" t="inlineStr">
-        <is>
-          <t>SGMB Code</t>
-        </is>
-      </c>
-      <c r="B5" s="82" t="inlineStr">
-        <is>
-          <t>Workshop Name</t>
-        </is>
-      </c>
-      <c r="C5" s="83" t="inlineStr">
-        <is>
-          <t>اسم الورشة</t>
-        </is>
-      </c>
-      <c r="D5" s="82" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E5" s="77" t="inlineStr">
-        <is>
-          <t>Market Min</t>
-        </is>
-      </c>
-      <c r="F5" s="77" t="inlineStr">
-        <is>
-          <t>Market Median</t>
-        </is>
-      </c>
-      <c r="G5" s="77" t="inlineStr">
-        <is>
-          <t>Market Max</t>
-        </is>
-      </c>
-      <c r="H5" s="84" t="inlineStr">
-        <is>
-          <t>Online Class</t>
-        </is>
-      </c>
-      <c r="I5" s="85" t="inlineStr">
-        <is>
-          <t>One-Day Workshop</t>
-        </is>
-      </c>
-      <c r="J5" s="78" t="inlineStr">
-        <is>
-          <t>Full Course</t>
-        </is>
-      </c>
-      <c r="K5" s="82" t="inlineStr">
-        <is>
-          <t>Full Course Hrs</t>
-        </is>
-      </c>
-      <c r="L5" s="82" t="inlineStr">
-        <is>
-          <t>Notes</t>
+    <row r="5" ht="46" customHeight="1" s="27">
+      <c r="A5" s="90" t="inlineStr">
+        <is>
+          <t>SGMB Code
+رمز الورشة</t>
+        </is>
+      </c>
+      <c r="B5" s="90" t="inlineStr">
+        <is>
+          <t>Workshop Name
+اسم الورشة (إنجليزي)</t>
+        </is>
+      </c>
+      <c r="C5" s="90" t="inlineStr">
+        <is>
+          <t>اسم الورشة
+Workshop (Arabic)</t>
+        </is>
+      </c>
+      <c r="D5" s="90" t="inlineStr">
+        <is>
+          <t>Category
+الفئة</t>
+        </is>
+      </c>
+      <c r="E5" s="91" t="inlineStr">
+        <is>
+          <t>Market Min
+أدنى سعر</t>
+        </is>
+      </c>
+      <c r="F5" s="91" t="inlineStr">
+        <is>
+          <t>Market Median
+متوسط السوق</t>
+        </is>
+      </c>
+      <c r="G5" s="91" t="inlineStr">
+        <is>
+          <t>Market Max
+أعلى سعر</t>
+        </is>
+      </c>
+      <c r="H5" s="92" t="inlineStr">
+        <is>
+          <t>Online Class
+الصف الإلكتروني</t>
+        </is>
+      </c>
+      <c r="I5" s="93" t="inlineStr">
+        <is>
+          <t>One-Day Workshop
+ورشة ليوم واحد</t>
+        </is>
+      </c>
+      <c r="J5" s="94" t="inlineStr">
+        <is>
+          <t>Full Course
+الدورة الكاملة</t>
+        </is>
+      </c>
+      <c r="K5" s="90" t="inlineStr">
+        <is>
+          <t>Full Course Hrs
+ساعات الدورة</t>
+        </is>
+      </c>
+      <c r="L5" s="90" t="inlineStr">
+        <is>
+          <t>Notes
+ملاحظات</t>
         </is>
       </c>
     </row>
@@ -1834,9 +1923,10 @@
           <t>ورشة أصول التعامل الإعلامي</t>
         </is>
       </c>
-      <c r="D6" s="37" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D6" s="89" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E6" s="38" t="n">
@@ -1878,9 +1968,10 @@
           <t>ورشة الصحافة الرقمية</t>
         </is>
       </c>
-      <c r="D7" s="43" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D7" s="88" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E7" s="44" t="n">
@@ -1922,9 +2013,10 @@
           <t>ورشة التقرير التلفزيوني</t>
         </is>
       </c>
-      <c r="D8" s="37" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D8" s="89" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E8" s="38" t="n">
@@ -1970,9 +2062,10 @@
           <t>ورشة مسار المقابلات الوظيفية</t>
         </is>
       </c>
-      <c r="D9" s="43" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D9" s="88" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E9" s="44" t="n">
@@ -2018,9 +2111,10 @@
           <t>ورشة فن الإدارة</t>
         </is>
       </c>
-      <c r="D10" s="37" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D10" s="89" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E10" s="38" t="n">
@@ -2062,9 +2156,10 @@
           <t>الورشة الصحفية</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D11" s="88" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E11" s="44" t="n">
@@ -2106,9 +2201,10 @@
           <t>ورشة تنظيم المنتديات الدولية</t>
         </is>
       </c>
-      <c r="D12" s="37" t="inlineStr">
-        <is>
-          <t>Events &amp; Protocol</t>
+      <c r="D12" s="89" t="inlineStr">
+        <is>
+          <t>Events &amp; Protocol
+الفعاليات والبروتوكول</t>
         </is>
       </c>
       <c r="E12" s="38" t="n">
@@ -2150,9 +2246,10 @@
           <t>ورشة المخاطبات الرسمية بالبريد الإلكتروني</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D13" s="88" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E13" s="44" t="n">
@@ -2194,9 +2291,10 @@
           <t>ورشة تنظيم الفعاليات</t>
         </is>
       </c>
-      <c r="D14" s="37" t="inlineStr">
-        <is>
-          <t>Events &amp; Protocol</t>
+      <c r="D14" s="89" t="inlineStr">
+        <is>
+          <t>Events &amp; Protocol
+الفعاليات والبروتوكول</t>
         </is>
       </c>
       <c r="E14" s="38" t="n">
@@ -2238,9 +2336,10 @@
           <t>ورشة التشريفات والبروتوكول</t>
         </is>
       </c>
-      <c r="D15" s="43" t="inlineStr">
-        <is>
-          <t>Events &amp; Protocol</t>
+      <c r="D15" s="88" t="inlineStr">
+        <is>
+          <t>Events &amp; Protocol
+الفعاليات والبروتوكول</t>
         </is>
       </c>
       <c r="E15" s="44" t="n">
@@ -2282,9 +2381,10 @@
           <t>ورشة التغطية الإعلامية لوسائل التواصل الاجتماعي</t>
         </is>
       </c>
-      <c r="D16" s="37" t="inlineStr">
-        <is>
-          <t>Social Media &amp; Digital</t>
+      <c r="D16" s="89" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital
+التواصل الاجتماعي والرقمي</t>
         </is>
       </c>
       <c r="E16" s="38" t="n">
@@ -2326,9 +2426,10 @@
           <t>ورشة التصوير الصحفي والفوتوغرافي</t>
         </is>
       </c>
-      <c r="D17" s="43" t="inlineStr">
-        <is>
-          <t>Design &amp; Photography</t>
+      <c r="D17" s="88" t="inlineStr">
+        <is>
+          <t>Design &amp; Photography
+التصميم والتصوير</t>
         </is>
       </c>
       <c r="E17" s="44" t="n">
@@ -2370,9 +2471,10 @@
           <t>ورشة تصوير البورتريه</t>
         </is>
       </c>
-      <c r="D18" s="37" t="inlineStr">
-        <is>
-          <t>Design &amp; Photography</t>
+      <c r="D18" s="89" t="inlineStr">
+        <is>
+          <t>Design &amp; Photography
+التصميم والتصوير</t>
         </is>
       </c>
       <c r="E18" s="38" t="n">
@@ -2414,9 +2516,10 @@
           <t>Workshop telling Story</t>
         </is>
       </c>
-      <c r="D19" s="43" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D19" s="88" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E19" s="44" t="n">
@@ -2458,9 +2561,10 @@
           <t>ورشة التغطيات الإعلامية</t>
         </is>
       </c>
-      <c r="D20" s="37" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D20" s="89" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E20" s="38" t="n">
@@ -2502,9 +2606,10 @@
           <t>ورشة القانون في مجال العمل</t>
         </is>
       </c>
-      <c r="D21" s="43" t="inlineStr">
-        <is>
-          <t>Legal</t>
+      <c r="D21" s="88" t="inlineStr">
+        <is>
+          <t>Legal
+القانون</t>
         </is>
       </c>
       <c r="E21" s="44" t="n">
@@ -2546,9 +2651,10 @@
           <t>ورشة التفكير الإبداعي في مجال العمل</t>
         </is>
       </c>
-      <c r="D22" s="37" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D22" s="89" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E22" s="38" t="n">
@@ -2590,9 +2696,10 @@
           <t>ورشة الإخراج التلفزيوني</t>
         </is>
       </c>
-      <c r="D23" s="43" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D23" s="88" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E23" s="44" t="n">
@@ -2634,9 +2741,10 @@
           <t>ورشة المونتاج التلفزيوني</t>
         </is>
       </c>
-      <c r="D24" s="37" t="inlineStr">
-        <is>
-          <t>Media &amp; Journalism</t>
+      <c r="D24" s="89" t="inlineStr">
+        <is>
+          <t>Media &amp; Journalism
+الإعلام والصحافة</t>
         </is>
       </c>
       <c r="E24" s="38" t="n">
@@ -2682,9 +2790,10 @@
           <t>ورشة التحقق من المعلومات المنشورة على وسائل التواصل الاجتماعي</t>
         </is>
       </c>
-      <c r="D25" s="43" t="inlineStr">
-        <is>
-          <t>Social Media &amp; Digital</t>
+      <c r="D25" s="88" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital
+التواصل الاجتماعي والرقمي</t>
         </is>
       </c>
       <c r="E25" s="44" t="n">
@@ -2730,9 +2839,10 @@
           <t>ورشة تنسيق وتصميم الجرافيك لوسائل التواصل الاجتماعي</t>
         </is>
       </c>
-      <c r="D26" s="37" t="inlineStr">
-        <is>
-          <t>Social Media &amp; Digital</t>
+      <c r="D26" s="89" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital
+التواصل الاجتماعي والرقمي</t>
         </is>
       </c>
       <c r="E26" s="38" t="n">
@@ -2774,9 +2884,10 @@
           <t>ورشة تصميم الجرافيك</t>
         </is>
       </c>
-      <c r="D27" s="43" t="inlineStr">
-        <is>
-          <t>Design &amp; Photography</t>
+      <c r="D27" s="88" t="inlineStr">
+        <is>
+          <t>Design &amp; Photography
+التصميم والتصوير</t>
         </is>
       </c>
       <c r="E27" s="44" t="n">
@@ -2818,9 +2929,10 @@
           <t>ورشة الاتصال الاستراتيجي</t>
         </is>
       </c>
-      <c r="D28" s="37" t="inlineStr">
-        <is>
-          <t>Social Media &amp; Digital</t>
+      <c r="D28" s="89" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Digital
+التواصل الاجتماعي والرقمي</t>
         </is>
       </c>
       <c r="E28" s="38" t="n">
@@ -2862,9 +2974,10 @@
           <t>ورشة إدارة محتوى المواقع الإلكترونية</t>
         </is>
       </c>
-      <c r="D29" s="43" t="inlineStr">
-        <is>
-          <t>Technology &amp; Cybersecurity</t>
+      <c r="D29" s="88" t="inlineStr">
+        <is>
+          <t>Technology &amp; Cybersecurity
+التقنية والأمن السيبراني</t>
         </is>
       </c>
       <c r="E29" s="44" t="n">
@@ -2910,9 +3023,10 @@
           <t>ورشة الموازنات المالية</t>
         </is>
       </c>
-      <c r="D30" s="37" t="inlineStr">
-        <is>
-          <t>Management &amp; Professional</t>
+      <c r="D30" s="89" t="inlineStr">
+        <is>
+          <t>Management &amp; Professional
+الإدارة والمهارات المهنية</t>
         </is>
       </c>
       <c r="E30" s="38" t="n">
@@ -2954,9 +3068,10 @@
           <t>ورشة مهارات استخدام تطبيقات الحاسوب</t>
         </is>
       </c>
-      <c r="D31" s="43" t="inlineStr">
-        <is>
-          <t>Technology &amp; Cybersecurity</t>
+      <c r="D31" s="88" t="inlineStr">
+        <is>
+          <t>Technology &amp; Cybersecurity
+التقنية والأمن السيبراني</t>
         </is>
       </c>
       <c r="E31" s="44" t="n">
@@ -3002,9 +3117,10 @@
           <t>ورشة الوقاية والحماية من الاختراقات</t>
         </is>
       </c>
-      <c r="D32" s="37" t="inlineStr">
-        <is>
-          <t>Technology &amp; Cybersecurity</t>
+      <c r="D32" s="89" t="inlineStr">
+        <is>
+          <t>Technology &amp; Cybersecurity
+التقنية والأمن السيبراني</t>
         </is>
       </c>
       <c r="E32" s="38" t="n">

</xml_diff>